<commit_message>
Added info to tab Feb
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inbetgroup-my.sharepoint.com/personal/adriana_koleva_inbet_com/Documents/Projects/CRM/Promos/Promo Calendars/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inbetgroup-my.sharepoint.com/personal/adriana_koleva_inbet_com/Documents/Projects/GitHubPromoCalendar/promo_calendar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A054E8F-7224-4C51-B56C-9E116527A6E3}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7CEC7DC-7D13-42AB-9107-8EAA1B1B1018}"/>
   <bookViews>
-    <workbookView xWindow="-14055" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Януари26" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="168">
   <si>
     <t>CASINO March 2026</t>
   </si>
@@ -985,41 +985,173 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1027,13 +1159,64 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1042,34 +1225,22 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1084,193 +1255,22 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1288,10 +1288,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1560,9 +1556,515 @@
   <sheetPr>
     <tabColor theme="5" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="37.799999999999997" x14ac:dyDescent="0.3">
+      <c r="A1" s="74" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+    </row>
+    <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
+        <v>23</v>
+      </c>
+      <c r="B3" s="5">
+        <v>24</v>
+      </c>
+      <c r="C3" s="5">
+        <v>25</v>
+      </c>
+      <c r="D3" s="5">
+        <v>26</v>
+      </c>
+      <c r="E3" s="5">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
+        <v>28</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A6" s="103" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="104"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="106" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="107"/>
+      <c r="F6" s="107"/>
+      <c r="G6" s="107"/>
+    </row>
+    <row r="7" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A7" s="110" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="110" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="112" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A8" s="111"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="113"/>
+      <c r="E8" s="123" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="124"/>
+      <c r="G8" s="125"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="20">
+        <v>10</v>
+      </c>
+      <c r="C10" s="20">
+        <v>11</v>
+      </c>
+      <c r="D10" s="20">
+        <v>12</v>
+      </c>
+      <c r="E10" s="20">
+        <v>13</v>
+      </c>
+      <c r="F10" s="20">
+        <v>14</v>
+      </c>
+      <c r="G10" s="20">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A11" s="103" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="105"/>
+      <c r="C11" s="121" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="122"/>
+      <c r="E11" s="122"/>
+      <c r="F11" s="122"/>
+      <c r="G11" s="122"/>
+    </row>
+    <row r="12" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A12" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A14" s="20">
+        <v>16</v>
+      </c>
+      <c r="B14" s="20">
+        <v>17</v>
+      </c>
+      <c r="C14" s="20">
+        <v>18</v>
+      </c>
+      <c r="D14" s="20">
+        <v>19</v>
+      </c>
+      <c r="E14" s="20">
+        <v>20</v>
+      </c>
+      <c r="F14" s="20">
+        <v>21</v>
+      </c>
+      <c r="G14" s="20">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A15" s="123" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="124"/>
+      <c r="C15" s="125"/>
+      <c r="D15" s="106" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="107"/>
+      <c r="F15" s="107"/>
+      <c r="G15" s="107"/>
+    </row>
+    <row r="16" spans="1:7" ht="104.4" x14ac:dyDescent="0.3">
+      <c r="A16" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="27" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A18" s="20">
+        <v>23</v>
+      </c>
+      <c r="B18" s="20">
+        <v>24</v>
+      </c>
+      <c r="C18" s="20">
+        <v>25</v>
+      </c>
+      <c r="D18" s="20">
+        <v>26</v>
+      </c>
+      <c r="E18" s="20">
+        <v>27</v>
+      </c>
+      <c r="F18" s="20">
+        <v>28</v>
+      </c>
+      <c r="G18" s="20">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A19" s="119" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="120"/>
+      <c r="C19" s="130"/>
+      <c r="D19" s="82" t="s">
+        <v>72</v>
+      </c>
+      <c r="E19" s="83"/>
+      <c r="F19" s="83"/>
+      <c r="G19" s="83"/>
+    </row>
+    <row r="20" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A20" s="69" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" s="131" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" s="69" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="133" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="G20" s="28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A21" s="70"/>
+      <c r="B21" s="132"/>
+      <c r="C21" s="70"/>
+      <c r="D21" s="134"/>
+      <c r="E21" s="123" t="s">
+        <v>29</v>
+      </c>
+      <c r="F21" s="124"/>
+      <c r="G21" s="124"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="G22" s="19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A23" s="20">
+        <v>30</v>
+      </c>
+      <c r="B23" s="20">
+        <v>31</v>
+      </c>
+      <c r="C23" s="5">
+        <v>1</v>
+      </c>
+      <c r="D23" s="5">
+        <v>2</v>
+      </c>
+      <c r="E23" s="5">
+        <v>3</v>
+      </c>
+      <c r="F23" s="5">
+        <v>4</v>
+      </c>
+      <c r="G23" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A24" s="103" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" s="105"/>
+      <c r="C24" s="136"/>
+      <c r="D24" s="136"/>
+      <c r="E24" s="136"/>
+      <c r="F24" s="136"/>
+      <c r="G24" s="136"/>
+    </row>
+    <row r="25" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A25" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25" s="137"/>
+      <c r="D25" s="137"/>
+      <c r="E25" s="137"/>
+      <c r="F25" s="137"/>
+      <c r="G25" s="137"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" s="137"/>
+      <c r="D26" s="137"/>
+      <c r="E26" s="137"/>
+      <c r="F26" s="137"/>
+      <c r="G26" s="137"/>
+    </row>
+  </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E8:G8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1604,25 +2106,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="46" t="s">
+      <c r="I1" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="47"/>
-      <c r="O1" s="47"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
+      <c r="M1" s="75"/>
+      <c r="N1" s="75"/>
+      <c r="O1" s="75"/>
       <c r="P1" s="1"/>
     </row>
     <row r="2" spans="1:16" ht="21" x14ac:dyDescent="0.3">
@@ -1786,42 +2288,42 @@
       <c r="P5" s="1"/>
     </row>
     <row r="6" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="103" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="94"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="82" t="s">
+      <c r="B6" s="104"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="106" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="83"/>
-      <c r="F6" s="83"/>
-      <c r="G6" s="83"/>
+      <c r="E6" s="107"/>
+      <c r="F6" s="107"/>
+      <c r="G6" s="107"/>
       <c r="H6" s="1"/>
-      <c r="I6" s="53" t="s">
+      <c r="I6" s="116" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="66" t="s">
+      <c r="J6" s="119" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="67"/>
-      <c r="L6" s="67"/>
-      <c r="M6" s="67"/>
-      <c r="N6" s="67"/>
-      <c r="O6" s="67"/>
+      <c r="K6" s="120"/>
+      <c r="L6" s="120"/>
+      <c r="M6" s="120"/>
+      <c r="N6" s="120"/>
+      <c r="O6" s="120"/>
       <c r="P6" s="1"/>
     </row>
     <row r="7" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A7" s="95" t="s">
+      <c r="A7" s="110" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="95" t="s">
+      <c r="B7" s="110" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="95" t="s">
+      <c r="C7" s="110" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="97" t="s">
+      <c r="D7" s="112" t="s">
         <v>25</v>
       </c>
       <c r="E7" s="14" t="s">
@@ -1834,7 +2336,7 @@
         <v>28</v>
       </c>
       <c r="H7" s="1"/>
-      <c r="I7" s="54"/>
+      <c r="I7" s="117"/>
       <c r="J7" s="15"/>
       <c r="K7" s="16"/>
       <c r="L7" s="16"/>
@@ -1844,33 +2346,33 @@
       <c r="P7" s="1"/>
     </row>
     <row r="8" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A8" s="96"/>
-      <c r="B8" s="96"/>
-      <c r="C8" s="96"/>
-      <c r="D8" s="98"/>
-      <c r="E8" s="62" t="s">
+      <c r="A8" s="111"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="113"/>
+      <c r="E8" s="123" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="63"/>
-      <c r="G8" s="81"/>
+      <c r="F8" s="124"/>
+      <c r="G8" s="125"/>
       <c r="H8" s="1"/>
-      <c r="I8" s="54"/>
-      <c r="J8" s="72" t="s">
+      <c r="I8" s="117"/>
+      <c r="J8" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="K8" s="72" t="s">
+      <c r="K8" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="L8" s="72" t="s">
+      <c r="L8" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="M8" s="72" t="s">
+      <c r="M8" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="N8" s="72" t="s">
+      <c r="N8" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="O8" s="72" t="s">
+      <c r="O8" s="69" t="s">
         <v>35</v>
       </c>
       <c r="P8" s="1"/>
@@ -1898,13 +2400,13 @@
         <v>37</v>
       </c>
       <c r="H9" s="1"/>
-      <c r="I9" s="71"/>
-      <c r="J9" s="73"/>
-      <c r="K9" s="73"/>
-      <c r="L9" s="73"/>
-      <c r="M9" s="73"/>
-      <c r="N9" s="73"/>
-      <c r="O9" s="73"/>
+      <c r="I9" s="118"/>
+      <c r="J9" s="70"/>
+      <c r="K9" s="70"/>
+      <c r="L9" s="70"/>
+      <c r="M9" s="70"/>
+      <c r="N9" s="70"/>
+      <c r="O9" s="70"/>
       <c r="P9" s="1"/>
     </row>
     <row r="10" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -1954,29 +2456,29 @@
       <c r="P10" s="1"/>
     </row>
     <row r="11" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A11" s="64" t="s">
+      <c r="A11" s="103" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="65"/>
-      <c r="C11" s="90" t="s">
+      <c r="B11" s="105"/>
+      <c r="C11" s="121" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="91"/>
-      <c r="E11" s="91"/>
-      <c r="F11" s="91"/>
-      <c r="G11" s="91"/>
+      <c r="D11" s="122"/>
+      <c r="E11" s="122"/>
+      <c r="F11" s="122"/>
+      <c r="G11" s="122"/>
       <c r="H11" s="1"/>
-      <c r="I11" s="53" t="s">
+      <c r="I11" s="116" t="s">
         <v>11</v>
       </c>
       <c r="J11" s="21"/>
       <c r="K11" s="21"/>
       <c r="L11" s="21"/>
-      <c r="M11" s="69" t="s">
+      <c r="M11" s="82" t="s">
         <v>40</v>
       </c>
-      <c r="N11" s="70"/>
-      <c r="O11" s="70"/>
+      <c r="N11" s="83"/>
+      <c r="O11" s="83"/>
       <c r="P11" s="1"/>
     </row>
     <row r="12" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -2002,15 +2504,15 @@
         <v>47</v>
       </c>
       <c r="H12" s="1"/>
-      <c r="I12" s="54"/>
-      <c r="J12" s="92" t="s">
+      <c r="I12" s="117"/>
+      <c r="J12" s="96" t="s">
         <v>48</v>
       </c>
-      <c r="K12" s="93"/>
-      <c r="L12" s="93"/>
-      <c r="M12" s="93"/>
-      <c r="N12" s="93"/>
-      <c r="O12" s="93"/>
+      <c r="K12" s="97"/>
+      <c r="L12" s="97"/>
+      <c r="M12" s="97"/>
+      <c r="N12" s="97"/>
+      <c r="O12" s="97"/>
       <c r="P12" s="24"/>
     </row>
     <row r="13" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -2036,7 +2538,7 @@
         <v>37</v>
       </c>
       <c r="H13" s="1"/>
-      <c r="I13" s="71"/>
+      <c r="I13" s="118"/>
       <c r="J13" s="25" t="s">
         <v>49</v>
       </c>
@@ -2104,29 +2606,29 @@
       <c r="P14" s="1"/>
     </row>
     <row r="15" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A15" s="62" t="s">
+      <c r="A15" s="123" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="81"/>
-      <c r="D15" s="82" t="s">
+      <c r="B15" s="124"/>
+      <c r="C15" s="125"/>
+      <c r="D15" s="106" t="s">
         <v>56</v>
       </c>
-      <c r="E15" s="83"/>
-      <c r="F15" s="83"/>
-      <c r="G15" s="83"/>
+      <c r="E15" s="107"/>
+      <c r="F15" s="107"/>
+      <c r="G15" s="107"/>
       <c r="H15" s="1"/>
-      <c r="I15" s="53" t="s">
+      <c r="I15" s="116" t="s">
         <v>11</v>
       </c>
-      <c r="J15" s="84" t="s">
+      <c r="J15" s="64" t="s">
         <v>57</v>
       </c>
-      <c r="K15" s="85"/>
-      <c r="L15" s="85"/>
-      <c r="M15" s="85"/>
-      <c r="N15" s="85"/>
-      <c r="O15" s="85"/>
+      <c r="K15" s="73"/>
+      <c r="L15" s="73"/>
+      <c r="M15" s="73"/>
+      <c r="N15" s="73"/>
+      <c r="O15" s="73"/>
       <c r="P15" s="1"/>
     </row>
     <row r="16" spans="1:16" ht="34.799999999999997" x14ac:dyDescent="0.3">
@@ -2152,23 +2654,23 @@
         <v>64</v>
       </c>
       <c r="H16" s="1"/>
-      <c r="I16" s="54"/>
-      <c r="J16" s="86" t="s">
+      <c r="I16" s="117"/>
+      <c r="J16" s="126" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="86" t="s">
+      <c r="K16" s="126" t="s">
         <v>66</v>
       </c>
-      <c r="L16" s="88" t="s">
+      <c r="L16" s="128" t="s">
         <v>67</v>
       </c>
-      <c r="M16" s="88" t="s">
+      <c r="M16" s="128" t="s">
         <v>68</v>
       </c>
-      <c r="N16" s="88" t="s">
+      <c r="N16" s="128" t="s">
         <v>69</v>
       </c>
-      <c r="O16" s="88" t="s">
+      <c r="O16" s="128" t="s">
         <v>70</v>
       </c>
       <c r="P16" s="1"/>
@@ -2196,13 +2698,13 @@
         <v>37</v>
       </c>
       <c r="H17" s="1"/>
-      <c r="I17" s="71"/>
-      <c r="J17" s="87"/>
-      <c r="K17" s="87"/>
-      <c r="L17" s="89"/>
-      <c r="M17" s="89"/>
-      <c r="N17" s="89"/>
-      <c r="O17" s="89"/>
+      <c r="I17" s="118"/>
+      <c r="J17" s="127"/>
+      <c r="K17" s="127"/>
+      <c r="L17" s="129"/>
+      <c r="M17" s="129"/>
+      <c r="N17" s="129"/>
+      <c r="O17" s="129"/>
       <c r="P17" s="1"/>
     </row>
     <row r="18" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -2252,42 +2754,42 @@
       <c r="P18" s="1"/>
     </row>
     <row r="19" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A19" s="66" t="s">
+      <c r="A19" s="119" t="s">
         <v>71</v>
       </c>
-      <c r="B19" s="67"/>
-      <c r="C19" s="68"/>
-      <c r="D19" s="69" t="s">
+      <c r="B19" s="120"/>
+      <c r="C19" s="130"/>
+      <c r="D19" s="82" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="70"/>
-      <c r="F19" s="70"/>
-      <c r="G19" s="70"/>
+      <c r="E19" s="83"/>
+      <c r="F19" s="83"/>
+      <c r="G19" s="83"/>
       <c r="H19" s="1"/>
-      <c r="I19" s="53" t="s">
+      <c r="I19" s="116" t="s">
         <v>11</v>
       </c>
-      <c r="J19" s="69" t="s">
+      <c r="J19" s="82" t="s">
         <v>73</v>
       </c>
-      <c r="K19" s="70"/>
-      <c r="L19" s="70"/>
-      <c r="M19" s="70"/>
-      <c r="N19" s="70"/>
-      <c r="O19" s="70"/>
+      <c r="K19" s="83"/>
+      <c r="L19" s="83"/>
+      <c r="M19" s="83"/>
+      <c r="N19" s="83"/>
+      <c r="O19" s="83"/>
       <c r="P19" s="1"/>
     </row>
     <row r="20" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A20" s="72" t="s">
+      <c r="A20" s="69" t="s">
         <v>74</v>
       </c>
-      <c r="B20" s="74" t="s">
+      <c r="B20" s="131" t="s">
         <v>75</v>
       </c>
-      <c r="C20" s="72" t="s">
+      <c r="C20" s="69" t="s">
         <v>76</v>
       </c>
-      <c r="D20" s="76" t="s">
+      <c r="D20" s="133" t="s">
         <v>77</v>
       </c>
       <c r="E20" s="28" t="s">
@@ -2300,45 +2802,45 @@
         <v>80</v>
       </c>
       <c r="H20" s="1"/>
-      <c r="I20" s="54"/>
-      <c r="J20" s="78" t="s">
+      <c r="I20" s="117"/>
+      <c r="J20" s="86" t="s">
         <v>81</v>
       </c>
-      <c r="K20" s="78" t="s">
+      <c r="K20" s="86" t="s">
         <v>82</v>
       </c>
-      <c r="L20" s="59" t="s">
+      <c r="L20" s="138" t="s">
         <v>83</v>
       </c>
-      <c r="M20" s="59" t="s">
+      <c r="M20" s="138" t="s">
         <v>84</v>
       </c>
-      <c r="N20" s="59" t="s">
+      <c r="N20" s="138" t="s">
         <v>85</v>
       </c>
-      <c r="O20" s="59" t="s">
+      <c r="O20" s="138" t="s">
         <v>86</v>
       </c>
       <c r="P20" s="1"/>
     </row>
     <row r="21" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A21" s="73"/>
-      <c r="B21" s="75"/>
-      <c r="C21" s="73"/>
-      <c r="D21" s="77"/>
-      <c r="E21" s="62" t="s">
+      <c r="A21" s="70"/>
+      <c r="B21" s="132"/>
+      <c r="C21" s="70"/>
+      <c r="D21" s="134"/>
+      <c r="E21" s="123" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="63"/>
-      <c r="G21" s="63"/>
+      <c r="F21" s="124"/>
+      <c r="G21" s="124"/>
       <c r="H21" s="1"/>
-      <c r="I21" s="54"/>
-      <c r="J21" s="79"/>
-      <c r="K21" s="79"/>
-      <c r="L21" s="60"/>
-      <c r="M21" s="60"/>
-      <c r="N21" s="60"/>
-      <c r="O21" s="60"/>
+      <c r="I21" s="117"/>
+      <c r="J21" s="135"/>
+      <c r="K21" s="135"/>
+      <c r="L21" s="139"/>
+      <c r="M21" s="139"/>
+      <c r="N21" s="139"/>
+      <c r="O21" s="139"/>
       <c r="P21" s="1"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
@@ -2364,13 +2866,13 @@
         <v>37</v>
       </c>
       <c r="H22" s="1"/>
-      <c r="I22" s="71"/>
-      <c r="J22" s="80"/>
-      <c r="K22" s="80"/>
-      <c r="L22" s="61"/>
-      <c r="M22" s="61"/>
-      <c r="N22" s="61"/>
-      <c r="O22" s="61"/>
+      <c r="I22" s="118"/>
+      <c r="J22" s="87"/>
+      <c r="K22" s="87"/>
+      <c r="L22" s="140"/>
+      <c r="M22" s="140"/>
+      <c r="N22" s="140"/>
+      <c r="O22" s="140"/>
       <c r="P22" s="1"/>
     </row>
     <row r="23" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -2420,27 +2922,27 @@
       <c r="P23" s="1"/>
     </row>
     <row r="24" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A24" s="64" t="s">
+      <c r="A24" s="103" t="s">
         <v>87</v>
       </c>
-      <c r="B24" s="65"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="51"/>
-      <c r="G24" s="51"/>
+      <c r="B24" s="105"/>
+      <c r="C24" s="136"/>
+      <c r="D24" s="136"/>
+      <c r="E24" s="136"/>
+      <c r="F24" s="136"/>
+      <c r="G24" s="136"/>
       <c r="H24" s="1"/>
-      <c r="I24" s="53" t="s">
+      <c r="I24" s="116" t="s">
         <v>11</v>
       </c>
-      <c r="J24" s="55" t="s">
+      <c r="J24" s="114" t="s">
         <v>88</v>
       </c>
-      <c r="K24" s="56"/>
-      <c r="L24" s="56"/>
-      <c r="M24" s="56"/>
-      <c r="N24" s="56"/>
-      <c r="O24" s="56"/>
+      <c r="K24" s="115"/>
+      <c r="L24" s="115"/>
+      <c r="M24" s="115"/>
+      <c r="N24" s="115"/>
+      <c r="O24" s="115"/>
       <c r="P24" s="1"/>
     </row>
     <row r="25" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -2450,29 +2952,29 @@
       <c r="B25" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="C25" s="52"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="52"/>
-      <c r="F25" s="52"/>
-      <c r="G25" s="52"/>
+      <c r="C25" s="137"/>
+      <c r="D25" s="137"/>
+      <c r="E25" s="137"/>
+      <c r="F25" s="137"/>
+      <c r="G25" s="137"/>
       <c r="H25" s="1"/>
-      <c r="I25" s="54"/>
-      <c r="J25" s="57" t="s">
+      <c r="I25" s="117"/>
+      <c r="J25" s="101" t="s">
         <v>91</v>
       </c>
-      <c r="K25" s="57" t="s">
+      <c r="K25" s="101" t="s">
         <v>92</v>
       </c>
-      <c r="L25" s="57" t="s">
+      <c r="L25" s="101" t="s">
         <v>93</v>
       </c>
-      <c r="M25" s="57" t="s">
+      <c r="M25" s="101" t="s">
         <v>94</v>
       </c>
-      <c r="N25" s="57" t="s">
+      <c r="N25" s="101" t="s">
         <v>95</v>
       </c>
-      <c r="O25" s="57" t="s">
+      <c r="O25" s="101" t="s">
         <v>96</v>
       </c>
       <c r="P25" s="1"/>
@@ -2484,19 +2986,19 @@
       <c r="B26" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
-      <c r="E26" s="52"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="52"/>
+      <c r="C26" s="137"/>
+      <c r="D26" s="137"/>
+      <c r="E26" s="137"/>
+      <c r="F26" s="137"/>
+      <c r="G26" s="137"/>
       <c r="H26" s="1"/>
-      <c r="I26" s="54"/>
-      <c r="J26" s="58"/>
-      <c r="K26" s="58"/>
-      <c r="L26" s="58"/>
-      <c r="M26" s="58"/>
-      <c r="N26" s="58"/>
-      <c r="O26" s="58"/>
+      <c r="I26" s="117"/>
+      <c r="J26" s="102"/>
+      <c r="K26" s="102"/>
+      <c r="L26" s="102"/>
+      <c r="M26" s="102"/>
+      <c r="N26" s="102"/>
+      <c r="O26" s="102"/>
       <c r="P26" s="1"/>
     </row>
     <row r="27" spans="1:16" ht="21" x14ac:dyDescent="0.3">
@@ -2536,25 +3038,25 @@
       <c r="P28" s="1"/>
     </row>
     <row r="29" spans="1:16" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A29" s="46" t="s">
+      <c r="A29" s="74" t="s">
         <v>97</v>
       </c>
-      <c r="B29" s="47"/>
-      <c r="C29" s="47"/>
-      <c r="D29" s="47"/>
-      <c r="E29" s="47"/>
-      <c r="F29" s="47"/>
-      <c r="G29" s="47"/>
+      <c r="B29" s="75"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="75"/>
+      <c r="E29" s="75"/>
+      <c r="F29" s="75"/>
+      <c r="G29" s="75"/>
       <c r="H29" s="1"/>
-      <c r="I29" s="46" t="s">
+      <c r="I29" s="74" t="s">
         <v>98</v>
       </c>
-      <c r="J29" s="47"/>
-      <c r="K29" s="47"/>
-      <c r="L29" s="47"/>
-      <c r="M29" s="47"/>
-      <c r="N29" s="47"/>
-      <c r="O29" s="47"/>
+      <c r="J29" s="75"/>
+      <c r="K29" s="75"/>
+      <c r="L29" s="75"/>
+      <c r="M29" s="75"/>
+      <c r="N29" s="75"/>
+      <c r="O29" s="75"/>
       <c r="P29" s="1"/>
     </row>
     <row r="30" spans="1:16" ht="21" x14ac:dyDescent="0.3">
@@ -2716,11 +3218,11 @@
     <row r="34" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A34" s="36"/>
       <c r="B34" s="36"/>
-      <c r="C34" s="48" t="s">
+      <c r="C34" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="D34" s="49"/>
-      <c r="E34" s="50"/>
+      <c r="D34" s="62"/>
+      <c r="E34" s="63"/>
       <c r="F34" s="36"/>
       <c r="G34" s="36"/>
       <c r="H34" s="1"/>
@@ -2782,11 +3284,11 @@
     <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" s="7"/>
       <c r="B36" s="7"/>
-      <c r="C36" s="48" t="s">
+      <c r="C36" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="D36" s="49"/>
-      <c r="E36" s="50"/>
+      <c r="D36" s="62"/>
+      <c r="E36" s="63"/>
       <c r="F36" s="37"/>
       <c r="G36" s="37"/>
       <c r="H36" s="1"/>
@@ -2848,11 +3350,11 @@
     <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" s="8"/>
       <c r="B38" s="7"/>
-      <c r="C38" s="48" t="s">
+      <c r="C38" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="D38" s="49"/>
-      <c r="E38" s="50"/>
+      <c r="D38" s="62"/>
+      <c r="E38" s="63"/>
       <c r="F38" s="38"/>
       <c r="G38" s="38"/>
       <c r="H38" s="1"/>
@@ -2914,11 +3416,11 @@
     <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="32"/>
       <c r="B40" s="32"/>
-      <c r="C40" s="48" t="s">
+      <c r="C40" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="D40" s="49"/>
-      <c r="E40" s="50"/>
+      <c r="D40" s="62"/>
+      <c r="E40" s="63"/>
       <c r="F40" s="34"/>
       <c r="G40" s="34"/>
       <c r="H40" s="1"/>
@@ -3052,9 +3554,9 @@
     <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" s="40"/>
       <c r="B46" s="40"/>
-      <c r="C46" s="45"/>
-      <c r="D46" s="45"/>
-      <c r="E46" s="45"/>
+      <c r="C46" s="60"/>
+      <c r="D46" s="60"/>
+      <c r="E46" s="60"/>
       <c r="F46" s="39"/>
       <c r="G46" s="39"/>
       <c r="H46" s="1"/>
@@ -3088,9 +3590,9 @@
     <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" s="39"/>
       <c r="B48" s="39"/>
-      <c r="C48" s="45"/>
-      <c r="D48" s="45"/>
-      <c r="E48" s="45"/>
+      <c r="C48" s="60"/>
+      <c r="D48" s="60"/>
+      <c r="E48" s="60"/>
       <c r="F48" s="42"/>
       <c r="G48" s="42"/>
       <c r="H48" s="1"/>
@@ -3124,9 +3626,9 @@
     <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" s="40"/>
       <c r="B50" s="39"/>
-      <c r="C50" s="45"/>
-      <c r="D50" s="45"/>
-      <c r="E50" s="45"/>
+      <c r="C50" s="60"/>
+      <c r="D50" s="60"/>
+      <c r="E50" s="60"/>
       <c r="F50" s="40"/>
       <c r="G50" s="40"/>
       <c r="H50" s="1"/>
@@ -3160,9 +3662,9 @@
     <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" s="40"/>
       <c r="B52" s="40"/>
-      <c r="C52" s="45"/>
-      <c r="D52" s="45"/>
-      <c r="E52" s="45"/>
+      <c r="C52" s="60"/>
+      <c r="D52" s="60"/>
+      <c r="E52" s="60"/>
       <c r="F52" s="24"/>
       <c r="G52" s="24"/>
       <c r="H52" s="1"/>
@@ -3177,6 +3679,61 @@
     </row>
   </sheetData>
   <mergeCells count="71">
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="I29:O29"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="I24:I26"/>
+    <mergeCell ref="J24:O24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="K25:K26"/>
+    <mergeCell ref="L25:L26"/>
+    <mergeCell ref="M25:M26"/>
+    <mergeCell ref="N25:N26"/>
+    <mergeCell ref="O25:O26"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="I19:I22"/>
+    <mergeCell ref="J19:O19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="J20:J22"/>
+    <mergeCell ref="K20:K22"/>
+    <mergeCell ref="L20:L22"/>
+    <mergeCell ref="M20:M22"/>
+    <mergeCell ref="N20:N22"/>
+    <mergeCell ref="O20:O22"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="I15:I17"/>
+    <mergeCell ref="J15:O15"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="M16:M17"/>
+    <mergeCell ref="N16:N17"/>
+    <mergeCell ref="O16:O17"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="I11:I13"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="J12:O12"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="I1:O1"/>
     <mergeCell ref="A6:C6"/>
@@ -3188,66 +3745,11 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="O8:O9"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="I11:I13"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="J12:O12"/>
     <mergeCell ref="E8:G8"/>
     <mergeCell ref="J8:J9"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="L8:L9"/>
     <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D15:G15"/>
-    <mergeCell ref="I15:I17"/>
-    <mergeCell ref="J15:O15"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="K16:K17"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="M16:M17"/>
-    <mergeCell ref="N16:N17"/>
-    <mergeCell ref="O16:O17"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="I19:I22"/>
-    <mergeCell ref="J19:O19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="J20:J22"/>
-    <mergeCell ref="K20:K22"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="L20:L22"/>
-    <mergeCell ref="M20:M22"/>
-    <mergeCell ref="N20:N22"/>
-    <mergeCell ref="O20:O22"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="I24:I26"/>
-    <mergeCell ref="J24:O24"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="K25:K26"/>
-    <mergeCell ref="L25:L26"/>
-    <mergeCell ref="M25:M26"/>
-    <mergeCell ref="N25:N26"/>
-    <mergeCell ref="O25:O26"/>
-    <mergeCell ref="I29:O29"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="A29:G29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3296,25 +3798,25 @@
       <c r="P1" s="1"/>
     </row>
     <row r="2" spans="1:16" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="74" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
+      <c r="B2" s="75"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="46" t="s">
+      <c r="I2" s="74" t="s">
         <v>101</v>
       </c>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="47"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="47"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="75"/>
+      <c r="M2" s="75"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="75"/>
       <c r="P2" s="1"/>
     </row>
     <row r="3" spans="1:16" ht="21" x14ac:dyDescent="0.3">
@@ -3412,63 +3914,63 @@
     <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
-      <c r="C5" s="72" t="s">
+      <c r="C5" s="69" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D5" s="82" t="s">
         <v>102</v>
       </c>
-      <c r="E5" s="70"/>
-      <c r="F5" s="70"/>
-      <c r="G5" s="70"/>
+      <c r="E5" s="83"/>
+      <c r="F5" s="83"/>
+      <c r="G5" s="83"/>
       <c r="H5" s="1"/>
-      <c r="I5" s="111" t="s">
+      <c r="I5" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="J5" s="55" t="s">
+      <c r="J5" s="114" t="s">
         <v>88</v>
       </c>
-      <c r="K5" s="56"/>
-      <c r="L5" s="56"/>
-      <c r="M5" s="56"/>
-      <c r="N5" s="56"/>
-      <c r="O5" s="56"/>
+      <c r="K5" s="115"/>
+      <c r="L5" s="115"/>
+      <c r="M5" s="115"/>
+      <c r="N5" s="115"/>
+      <c r="O5" s="115"/>
       <c r="P5" s="1"/>
     </row>
     <row r="6" spans="1:16" ht="34.799999999999997" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
-      <c r="C6" s="73"/>
+      <c r="C6" s="70"/>
       <c r="D6" s="28" t="s">
         <v>44</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>103</v>
       </c>
-      <c r="F6" s="99" t="s">
+      <c r="F6" s="45" t="s">
         <v>104</v>
       </c>
-      <c r="G6" s="99" t="s">
+      <c r="G6" s="45" t="s">
         <v>105</v>
       </c>
       <c r="H6" s="1"/>
-      <c r="I6" s="112"/>
-      <c r="J6" s="57" t="s">
+      <c r="I6" s="72"/>
+      <c r="J6" s="101" t="s">
         <v>91</v>
       </c>
-      <c r="K6" s="57" t="s">
+      <c r="K6" s="101" t="s">
         <v>92</v>
       </c>
-      <c r="L6" s="57" t="s">
+      <c r="L6" s="101" t="s">
         <v>93</v>
       </c>
-      <c r="M6" s="57" t="s">
+      <c r="M6" s="101" t="s">
         <v>94</v>
       </c>
-      <c r="N6" s="57" t="s">
+      <c r="N6" s="101" t="s">
         <v>95</v>
       </c>
-      <c r="O6" s="57" t="s">
+      <c r="O6" s="101" t="s">
         <v>96</v>
       </c>
       <c r="P6" s="1"/>
@@ -3496,13 +3998,13 @@
         <v>107</v>
       </c>
       <c r="H7" s="1"/>
-      <c r="I7" s="113"/>
-      <c r="J7" s="58"/>
-      <c r="K7" s="58"/>
-      <c r="L7" s="58"/>
-      <c r="M7" s="58"/>
-      <c r="N7" s="58"/>
-      <c r="O7" s="58"/>
+      <c r="I7" s="81"/>
+      <c r="J7" s="102"/>
+      <c r="K7" s="102"/>
+      <c r="L7" s="102"/>
+      <c r="M7" s="102"/>
+      <c r="N7" s="102"/>
+      <c r="O7" s="102"/>
       <c r="P7" s="1"/>
     </row>
     <row r="8" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -3552,42 +4054,42 @@
       <c r="P8" s="1"/>
     </row>
     <row r="9" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A9" s="64" t="s">
+      <c r="A9" s="103" t="s">
         <v>108</v>
       </c>
-      <c r="B9" s="94"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="82" t="s">
+      <c r="B9" s="104"/>
+      <c r="C9" s="105"/>
+      <c r="D9" s="106" t="s">
         <v>109</v>
       </c>
-      <c r="E9" s="83"/>
-      <c r="F9" s="83"/>
-      <c r="G9" s="83"/>
+      <c r="E9" s="107"/>
+      <c r="F9" s="107"/>
+      <c r="G9" s="107"/>
       <c r="H9" s="1"/>
-      <c r="I9" s="111" t="s">
+      <c r="I9" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="J9" s="64" t="s">
+      <c r="J9" s="103" t="s">
         <v>110</v>
       </c>
-      <c r="K9" s="94"/>
-      <c r="L9" s="94"/>
-      <c r="M9" s="94"/>
-      <c r="N9" s="94"/>
-      <c r="O9" s="94"/>
+      <c r="K9" s="104"/>
+      <c r="L9" s="104"/>
+      <c r="M9" s="104"/>
+      <c r="N9" s="104"/>
+      <c r="O9" s="104"/>
       <c r="P9" s="1"/>
     </row>
     <row r="10" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A10" s="114" t="s">
+      <c r="A10" s="108" t="s">
         <v>111</v>
       </c>
-      <c r="B10" s="114" t="s">
+      <c r="B10" s="108" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="95" t="s">
+      <c r="C10" s="110" t="s">
         <v>113</v>
       </c>
-      <c r="D10" s="97" t="s">
+      <c r="D10" s="112" t="s">
         <v>114</v>
       </c>
       <c r="E10" s="14" t="s">
@@ -3600,45 +4102,45 @@
         <v>117</v>
       </c>
       <c r="H10" s="1"/>
-      <c r="I10" s="112"/>
-      <c r="J10" s="116" t="s">
+      <c r="I10" s="72"/>
+      <c r="J10" s="98" t="s">
         <v>118</v>
       </c>
-      <c r="K10" s="116" t="s">
+      <c r="K10" s="98" t="s">
         <v>119</v>
       </c>
-      <c r="L10" s="116" t="s">
+      <c r="L10" s="98" t="s">
         <v>120</v>
       </c>
-      <c r="M10" s="116" t="s">
+      <c r="M10" s="98" t="s">
         <v>121</v>
       </c>
-      <c r="N10" s="116" t="s">
+      <c r="N10" s="98" t="s">
         <v>122</v>
       </c>
-      <c r="O10" s="116" t="s">
+      <c r="O10" s="98" t="s">
         <v>123</v>
       </c>
       <c r="P10" s="1"/>
     </row>
     <row r="11" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A11" s="115"/>
-      <c r="B11" s="115"/>
-      <c r="C11" s="96"/>
-      <c r="D11" s="98"/>
-      <c r="E11" s="119" t="s">
+      <c r="A11" s="109"/>
+      <c r="B11" s="109"/>
+      <c r="C11" s="111"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="88" t="s">
         <v>124</v>
       </c>
-      <c r="F11" s="120"/>
-      <c r="G11" s="120"/>
+      <c r="F11" s="89"/>
+      <c r="G11" s="89"/>
       <c r="H11" s="1"/>
-      <c r="I11" s="112"/>
-      <c r="J11" s="117"/>
-      <c r="K11" s="117"/>
-      <c r="L11" s="117"/>
-      <c r="M11" s="117"/>
-      <c r="N11" s="117"/>
-      <c r="O11" s="117"/>
+      <c r="I11" s="72"/>
+      <c r="J11" s="99"/>
+      <c r="K11" s="99"/>
+      <c r="L11" s="99"/>
+      <c r="M11" s="99"/>
+      <c r="N11" s="99"/>
+      <c r="O11" s="99"/>
       <c r="P11" s="1"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
@@ -3664,13 +4166,13 @@
         <v>107</v>
       </c>
       <c r="H12" s="1"/>
-      <c r="I12" s="113"/>
-      <c r="J12" s="118"/>
-      <c r="K12" s="118"/>
-      <c r="L12" s="118"/>
-      <c r="M12" s="118"/>
-      <c r="N12" s="118"/>
-      <c r="O12" s="118"/>
+      <c r="I12" s="81"/>
+      <c r="J12" s="100"/>
+      <c r="K12" s="100"/>
+      <c r="L12" s="100"/>
+      <c r="M12" s="100"/>
+      <c r="N12" s="100"/>
+      <c r="O12" s="100"/>
       <c r="P12" s="1"/>
     </row>
     <row r="13" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -3720,63 +4222,63 @@
       <c r="P13" s="1"/>
     </row>
     <row r="14" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A14" s="121" t="s">
+      <c r="A14" s="90" t="s">
         <v>125</v>
       </c>
-      <c r="B14" s="122"/>
-      <c r="C14" s="122"/>
-      <c r="D14" s="123"/>
-      <c r="E14" s="125" t="s">
+      <c r="B14" s="91"/>
+      <c r="C14" s="91"/>
+      <c r="D14" s="92"/>
+      <c r="E14" s="93" t="s">
         <v>126</v>
       </c>
-      <c r="F14" s="124"/>
-      <c r="G14" s="124"/>
+      <c r="F14" s="94"/>
+      <c r="G14" s="94"/>
       <c r="H14" s="1"/>
-      <c r="I14" s="111" t="s">
+      <c r="I14" s="71" t="s">
         <v>11</v>
       </c>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
-      <c r="M14" s="126" t="s">
+      <c r="M14" s="95" t="s">
         <v>127</v>
       </c>
-      <c r="N14" s="126"/>
-      <c r="O14" s="126"/>
+      <c r="N14" s="95"/>
+      <c r="O14" s="95"/>
       <c r="P14" s="1"/>
     </row>
     <row r="15" spans="1:16" ht="34.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A15" s="100" t="s">
+      <c r="A15" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="B15" s="100" t="s">
+      <c r="B15" s="46" t="s">
         <v>129</v>
       </c>
-      <c r="C15" s="101" t="s">
+      <c r="C15" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="100" t="s">
+      <c r="D15" s="46" t="s">
         <v>130</v>
       </c>
-      <c r="E15" s="102" t="s">
+      <c r="E15" s="48" t="s">
         <v>131</v>
       </c>
-      <c r="F15" s="103" t="s">
+      <c r="F15" s="49" t="s">
         <v>132</v>
       </c>
-      <c r="G15" s="103" t="s">
+      <c r="G15" s="49" t="s">
         <v>133</v>
       </c>
       <c r="H15" s="1"/>
-      <c r="I15" s="112"/>
-      <c r="J15" s="92" t="s">
+      <c r="I15" s="72"/>
+      <c r="J15" s="96" t="s">
         <v>134</v>
       </c>
-      <c r="K15" s="93"/>
-      <c r="L15" s="93"/>
-      <c r="M15" s="93"/>
-      <c r="N15" s="93"/>
-      <c r="O15" s="93"/>
+      <c r="K15" s="97"/>
+      <c r="L15" s="97"/>
+      <c r="M15" s="97"/>
+      <c r="N15" s="97"/>
+      <c r="O15" s="97"/>
       <c r="P15" s="1"/>
     </row>
     <row r="16" spans="1:16" ht="41.4" x14ac:dyDescent="0.3">
@@ -3802,23 +4304,23 @@
         <v>107</v>
       </c>
       <c r="H16" s="1"/>
-      <c r="I16" s="113"/>
-      <c r="J16" s="104" t="s">
+      <c r="I16" s="81"/>
+      <c r="J16" s="50" t="s">
         <v>135</v>
       </c>
-      <c r="K16" s="104" t="s">
+      <c r="K16" s="50" t="s">
         <v>136</v>
       </c>
-      <c r="L16" s="105" t="s">
+      <c r="L16" s="51" t="s">
         <v>137</v>
       </c>
-      <c r="M16" s="104" t="s">
+      <c r="M16" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="N16" s="105" t="s">
+      <c r="N16" s="51" t="s">
         <v>139</v>
       </c>
-      <c r="O16" s="104" t="s">
+      <c r="O16" s="50" t="s">
         <v>140</v>
       </c>
       <c r="P16" s="24"/>
@@ -3870,39 +4372,39 @@
       <c r="P17" s="1"/>
     </row>
     <row r="18" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A18" s="127" t="s">
+      <c r="A18" s="76" t="s">
         <v>141</v>
       </c>
-      <c r="B18" s="128"/>
-      <c r="C18" s="129"/>
-      <c r="D18" s="130" t="s">
+      <c r="B18" s="77"/>
+      <c r="C18" s="78"/>
+      <c r="D18" s="79" t="s">
         <v>142</v>
       </c>
-      <c r="E18" s="131"/>
-      <c r="F18" s="131"/>
-      <c r="G18" s="131"/>
+      <c r="E18" s="80"/>
+      <c r="F18" s="80"/>
+      <c r="G18" s="80"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="111" t="s">
+      <c r="I18" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="J18" s="69" t="s">
+      <c r="J18" s="82" t="s">
         <v>143</v>
       </c>
-      <c r="K18" s="70"/>
-      <c r="L18" s="70"/>
-      <c r="M18" s="70"/>
-      <c r="N18" s="70"/>
-      <c r="O18" s="70"/>
+      <c r="K18" s="83"/>
+      <c r="L18" s="83"/>
+      <c r="M18" s="83"/>
+      <c r="N18" s="83"/>
+      <c r="O18" s="83"/>
       <c r="P18" s="1"/>
     </row>
     <row r="19" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A19" s="106" t="s">
+      <c r="A19" s="52" t="s">
         <v>144</v>
       </c>
-      <c r="B19" s="106" t="s">
+      <c r="B19" s="52" t="s">
         <v>145</v>
       </c>
-      <c r="C19" s="106" t="s">
+      <c r="C19" s="52" t="s">
         <v>146</v>
       </c>
       <c r="D19" s="22" t="s">
@@ -3918,23 +4420,23 @@
         <v>150</v>
       </c>
       <c r="H19" s="1"/>
-      <c r="I19" s="112"/>
-      <c r="J19" s="132" t="s">
+      <c r="I19" s="72"/>
+      <c r="J19" s="84" t="s">
         <v>151</v>
       </c>
-      <c r="K19" s="132" t="s">
+      <c r="K19" s="84" t="s">
         <v>152</v>
       </c>
-      <c r="L19" s="78" t="s">
+      <c r="L19" s="86" t="s">
         <v>153</v>
       </c>
-      <c r="M19" s="78" t="s">
+      <c r="M19" s="86" t="s">
         <v>154</v>
       </c>
-      <c r="N19" s="78" t="s">
+      <c r="N19" s="86" t="s">
         <v>155</v>
       </c>
-      <c r="O19" s="78" t="s">
+      <c r="O19" s="86" t="s">
         <v>156</v>
       </c>
       <c r="P19" s="1"/>
@@ -3962,13 +4464,13 @@
         <v>107</v>
       </c>
       <c r="H20" s="1"/>
-      <c r="I20" s="113"/>
-      <c r="J20" s="133"/>
-      <c r="K20" s="133"/>
-      <c r="L20" s="80"/>
-      <c r="M20" s="80"/>
-      <c r="N20" s="80"/>
-      <c r="O20" s="80"/>
+      <c r="I20" s="81"/>
+      <c r="J20" s="85"/>
+      <c r="K20" s="85"/>
+      <c r="L20" s="87"/>
+      <c r="M20" s="87"/>
+      <c r="N20" s="87"/>
+      <c r="O20" s="87"/>
       <c r="P20" s="1"/>
     </row>
     <row r="21" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -3984,13 +4486,13 @@
       <c r="D21" s="20">
         <v>30</v>
       </c>
-      <c r="E21" s="107" t="s">
+      <c r="E21" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="F21" s="107" t="s">
+      <c r="F21" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="G21" s="107" t="s">
+      <c r="G21" s="53" t="s">
         <v>13</v>
       </c>
       <c r="H21" s="1"/>
@@ -4006,75 +4508,75 @@
       <c r="L21" s="20">
         <v>30</v>
       </c>
-      <c r="M21" s="107" t="s">
+      <c r="M21" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="N21" s="107" t="s">
+      <c r="N21" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="O21" s="107" t="s">
+      <c r="O21" s="53" t="s">
         <v>13</v>
       </c>
       <c r="P21" s="1"/>
     </row>
     <row r="22" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A22" s="134" t="s">
+      <c r="A22" s="66" t="s">
         <v>157</v>
       </c>
-      <c r="B22" s="135"/>
-      <c r="C22" s="136"/>
-      <c r="D22" s="72" t="s">
+      <c r="B22" s="67"/>
+      <c r="C22" s="68"/>
+      <c r="D22" s="69" t="s">
         <v>10</v>
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
       <c r="H22" s="1"/>
-      <c r="I22" s="111" t="s">
+      <c r="I22" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="J22" s="84" t="s">
+      <c r="J22" s="64" t="s">
         <v>158</v>
       </c>
-      <c r="K22" s="85"/>
-      <c r="L22" s="85"/>
-      <c r="M22" s="85"/>
-      <c r="N22" s="85"/>
-      <c r="O22" s="85"/>
+      <c r="K22" s="73"/>
+      <c r="L22" s="73"/>
+      <c r="M22" s="73"/>
+      <c r="N22" s="73"/>
+      <c r="O22" s="73"/>
       <c r="P22" s="1"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A23" s="108" t="s">
+      <c r="A23" s="54" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="108" t="s">
+      <c r="B23" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="C23" s="108" t="s">
+      <c r="C23" s="54" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="73"/>
+      <c r="D23" s="70"/>
       <c r="E23" s="34"/>
       <c r="F23" s="34"/>
       <c r="G23" s="34"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="112"/>
-      <c r="J23" s="109" t="s">
+      <c r="I23" s="72"/>
+      <c r="J23" s="55" t="s">
         <v>159</v>
       </c>
-      <c r="K23" s="109" t="s">
+      <c r="K23" s="55" t="s">
         <v>160</v>
       </c>
-      <c r="L23" s="110" t="s">
+      <c r="L23" s="56" t="s">
         <v>161</v>
       </c>
-      <c r="M23" s="110" t="s">
+      <c r="M23" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="N23" s="110" t="s">
+      <c r="N23" s="56" t="s">
         <v>163</v>
       </c>
-      <c r="O23" s="110" t="s">
+      <c r="O23" s="56" t="s">
         <v>164</v>
       </c>
       <c r="P23" s="1"/>
@@ -4124,25 +4626,25 @@
       <c r="P25" s="1"/>
     </row>
     <row r="26" spans="1:16" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A26" s="46" t="s">
+      <c r="A26" s="74" t="s">
         <v>165</v>
       </c>
-      <c r="B26" s="47"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="47"/>
-      <c r="E26" s="47"/>
-      <c r="F26" s="47"/>
-      <c r="G26" s="47"/>
+      <c r="B26" s="75"/>
+      <c r="C26" s="75"/>
+      <c r="D26" s="75"/>
+      <c r="E26" s="75"/>
+      <c r="F26" s="75"/>
+      <c r="G26" s="75"/>
       <c r="H26" s="1"/>
-      <c r="I26" s="46" t="s">
+      <c r="I26" s="74" t="s">
         <v>166</v>
       </c>
-      <c r="J26" s="47"/>
-      <c r="K26" s="47"/>
-      <c r="L26" s="47"/>
-      <c r="M26" s="47"/>
-      <c r="N26" s="47"/>
-      <c r="O26" s="47"/>
+      <c r="J26" s="75"/>
+      <c r="K26" s="75"/>
+      <c r="L26" s="75"/>
+      <c r="M26" s="75"/>
+      <c r="N26" s="75"/>
+      <c r="O26" s="75"/>
       <c r="P26" s="1"/>
     </row>
     <row r="27" spans="1:16" ht="21" x14ac:dyDescent="0.3">
@@ -4240,11 +4742,11 @@
     <row r="29" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
-      <c r="C29" s="48" t="s">
+      <c r="C29" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="D29" s="49"/>
-      <c r="E29" s="50"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="63"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
       <c r="H29" s="35"/>
@@ -4304,17 +4806,17 @@
       <c r="P30" s="1"/>
     </row>
     <row r="31" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A31" s="84" t="s">
+      <c r="A31" s="64" t="s">
         <v>167</v>
       </c>
-      <c r="B31" s="140"/>
-      <c r="C31" s="137"/>
-      <c r="D31" s="137"/>
-      <c r="E31" s="48" t="s">
+      <c r="B31" s="65"/>
+      <c r="C31" s="57"/>
+      <c r="D31" s="57"/>
+      <c r="E31" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="F31" s="49"/>
-      <c r="G31" s="49"/>
+      <c r="F31" s="62"/>
+      <c r="G31" s="62"/>
       <c r="H31" s="1"/>
       <c r="I31" s="36"/>
       <c r="J31" s="36"/>
@@ -4374,11 +4876,11 @@
     <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="7"/>
       <c r="B33" s="7"/>
-      <c r="C33" s="48" t="s">
+      <c r="C33" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="D33" s="49"/>
-      <c r="E33" s="50"/>
+      <c r="D33" s="62"/>
+      <c r="E33" s="63"/>
       <c r="F33" s="37"/>
       <c r="G33" s="37"/>
       <c r="H33" s="1"/>
@@ -4438,15 +4940,15 @@
       <c r="P34" s="1"/>
     </row>
     <row r="35" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A35" s="138"/>
-      <c r="B35" s="139"/>
-      <c r="C35" s="48" t="s">
+      <c r="A35" s="58"/>
+      <c r="B35" s="59"/>
+      <c r="C35" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="D35" s="49"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="137"/>
-      <c r="G35" s="137"/>
+      <c r="D35" s="62"/>
+      <c r="E35" s="63"/>
+      <c r="F35" s="57"/>
+      <c r="G35" s="57"/>
       <c r="H35" s="1"/>
       <c r="I35" s="8"/>
       <c r="J35" s="7"/>
@@ -4470,13 +4972,13 @@
       <c r="D36" s="20">
         <v>30</v>
       </c>
-      <c r="E36" s="107" t="s">
+      <c r="E36" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="F36" s="107" t="s">
+      <c r="F36" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="107" t="s">
+      <c r="G36" s="53" t="s">
         <v>13</v>
       </c>
       <c r="H36" s="1"/>
@@ -4492,22 +4994,22 @@
       <c r="L36" s="20">
         <v>30</v>
       </c>
-      <c r="M36" s="107" t="s">
+      <c r="M36" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="N36" s="107" t="s">
+      <c r="N36" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="O36" s="107" t="s">
+      <c r="O36" s="53" t="s">
         <v>13</v>
       </c>
       <c r="P36" s="1"/>
     </row>
     <row r="37" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A37" s="84" t="s">
+      <c r="A37" s="64" t="s">
         <v>167</v>
       </c>
-      <c r="B37" s="140"/>
+      <c r="B37" s="65"/>
       <c r="C37" s="36"/>
       <c r="D37" s="36"/>
       <c r="E37" s="36"/>
@@ -4580,9 +5082,9 @@
     <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="40"/>
       <c r="B41" s="40"/>
-      <c r="C41" s="45"/>
-      <c r="D41" s="45"/>
-      <c r="E41" s="45"/>
+      <c r="C41" s="60"/>
+      <c r="D41" s="60"/>
+      <c r="E41" s="60"/>
       <c r="F41" s="39"/>
       <c r="G41" s="39"/>
       <c r="H41" s="1"/>
@@ -4616,9 +5118,9 @@
     <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" s="39"/>
       <c r="B43" s="39"/>
-      <c r="C43" s="45"/>
-      <c r="D43" s="45"/>
-      <c r="E43" s="45"/>
+      <c r="C43" s="60"/>
+      <c r="D43" s="60"/>
+      <c r="E43" s="60"/>
       <c r="F43" s="42"/>
       <c r="G43" s="42"/>
       <c r="H43" s="1"/>
@@ -4652,9 +5154,9 @@
     <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" s="40"/>
       <c r="B45" s="39"/>
-      <c r="C45" s="45"/>
-      <c r="D45" s="45"/>
-      <c r="E45" s="45"/>
+      <c r="C45" s="60"/>
+      <c r="D45" s="60"/>
+      <c r="E45" s="60"/>
       <c r="F45" s="40"/>
       <c r="G45" s="40"/>
       <c r="H45" s="1"/>
@@ -4688,9 +5190,9 @@
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" s="40"/>
       <c r="B47" s="40"/>
-      <c r="C47" s="45"/>
-      <c r="D47" s="45"/>
-      <c r="E47" s="45"/>
+      <c r="C47" s="60"/>
+      <c r="D47" s="60"/>
+      <c r="E47" s="60"/>
       <c r="F47" s="24"/>
       <c r="G47" s="24"/>
       <c r="H47" s="1"/>
@@ -4705,32 +5207,26 @@
     </row>
   </sheetData>
   <mergeCells count="58">
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="J22:O22"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="I26:O26"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="I18:I20"/>
-    <mergeCell ref="J18:O18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="I2:O2"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="J5:O5"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="O6:O7"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="I9:I12"/>
+    <mergeCell ref="J9:O9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="A14:D14"/>
     <mergeCell ref="E14:G14"/>
@@ -4743,26 +5239,32 @@
     <mergeCell ref="M10:M12"/>
     <mergeCell ref="N10:N12"/>
     <mergeCell ref="O10:O12"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="O6:O7"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="I9:I12"/>
-    <mergeCell ref="J9:O9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="I2:O2"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:G5"/>
-    <mergeCell ref="I5:I7"/>
-    <mergeCell ref="J5:O5"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="I18:I20"/>
+    <mergeCell ref="J18:O18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="J22:O22"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="I26:O26"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="C29:E29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>